<commit_message>
Linked data catalogue in the index page
</commit_message>
<xml_diff>
--- a/administrative-database-guidance/data/tbl_final_mapping.xlsx
+++ b/administrative-database-guidance/data/tbl_final_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MikaylaBoginsky\Documents\technicalguide\administrative-database-guidance\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D554B62-4C14-4B50-BFF3-3ACB9E61F549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BDCBA0C-E7B2-4A07-B942-A4497941A7C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="63555" yWindow="6165" windowWidth="22590" windowHeight="12195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="62655" yWindow="6630" windowWidth="22590" windowHeight="12195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="New Administrative Mapping" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="55">
   <si>
     <t xml:space="preserve">NPD </t>
   </si>
@@ -145,9 +145,6 @@
   </si>
   <si>
     <t xml:space="preserve">Predicted Grade </t>
-  </si>
-  <si>
-    <t>N</t>
   </si>
   <si>
     <t>Number of UCAS applications</t>
@@ -582,10 +579,10 @@
   <sheetData>
     <row r="1" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>0</v>
@@ -602,7 +599,7 @@
     </row>
     <row r="2" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>4</v>
@@ -622,7 +619,7 @@
     </row>
     <row r="3" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>8</v>
@@ -642,7 +639,7 @@
     </row>
     <row r="4" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>9</v>
@@ -662,7 +659,7 @@
     </row>
     <row r="5" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>10</v>
@@ -682,7 +679,7 @@
     </row>
     <row r="6" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>11</v>
@@ -702,7 +699,7 @@
     </row>
     <row r="7" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>12</v>
@@ -722,7 +719,7 @@
     </row>
     <row r="8" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>14</v>
@@ -742,7 +739,7 @@
     </row>
     <row r="9" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>15</v>
@@ -762,7 +759,7 @@
     </row>
     <row r="10" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>16</v>
@@ -782,7 +779,7 @@
     </row>
     <row r="11" spans="1:6" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B11" s="4" t="s">
         <v>17</v>
@@ -802,7 +799,7 @@
     </row>
     <row r="12" spans="1:6" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>18</v>
@@ -822,7 +819,7 @@
     </row>
     <row r="13" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B13" s="4" t="s">
         <v>19</v>
@@ -842,7 +839,7 @@
     </row>
     <row r="14" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B14" s="4" t="s">
         <v>20</v>
@@ -862,7 +859,7 @@
     </row>
     <row r="15" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B15" s="4" t="s">
         <v>21</v>
@@ -882,7 +879,7 @@
     </row>
     <row r="16" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>22</v>
@@ -902,7 +899,7 @@
     </row>
     <row r="17" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>23</v>
@@ -922,7 +919,7 @@
     </row>
     <row r="18" spans="1:6" ht="51.75" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B18" s="4" t="s">
         <v>24</v>
@@ -942,7 +939,7 @@
     </row>
     <row r="19" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B19" s="4" t="s">
         <v>25</v>
@@ -962,7 +959,7 @@
     </row>
     <row r="20" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A20" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B20" s="4" t="s">
         <v>26</v>
@@ -982,7 +979,7 @@
     </row>
     <row r="21" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A21" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B21" s="4" t="s">
         <v>27</v>
@@ -1002,7 +999,7 @@
     </row>
     <row r="22" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A22" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>28</v>
@@ -1022,7 +1019,7 @@
     </row>
     <row r="23" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A23" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>29</v>
@@ -1042,7 +1039,7 @@
     </row>
     <row r="24" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A24" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B24" s="4" t="s">
         <v>30</v>
@@ -1062,7 +1059,7 @@
     </row>
     <row r="25" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A25" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>31</v>
@@ -1082,7 +1079,7 @@
     </row>
     <row r="26" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B26" s="4" t="s">
         <v>32</v>
@@ -1102,7 +1099,7 @@
     </row>
     <row r="27" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>33</v>
@@ -1122,7 +1119,7 @@
     </row>
     <row r="28" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A28" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>34</v>
@@ -1142,7 +1139,7 @@
     </row>
     <row r="29" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B29" s="4" t="s">
         <v>35</v>
@@ -1162,7 +1159,7 @@
     </row>
     <row r="30" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A30" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B30" s="4" t="s">
         <v>36</v>
@@ -1182,7 +1179,7 @@
     </row>
     <row r="31" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A31" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>37</v>
@@ -1202,7 +1199,7 @@
     </row>
     <row r="32" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A32" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B32" s="4" t="s">
         <v>38</v>
@@ -1222,13 +1219,13 @@
     </row>
     <row r="33" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A33" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>39</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>6</v>
@@ -1242,10 +1239,10 @@
     </row>
     <row r="34" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>13</v>
@@ -1262,10 +1259,10 @@
     </row>
     <row r="35" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A35" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>13</v>
@@ -1282,10 +1279,10 @@
     </row>
     <row r="36" spans="1:6" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C36" s="11" t="s">
         <v>13</v>
@@ -1302,10 +1299,10 @@
     </row>
     <row r="37" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A37" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C37" s="11" t="s">
         <v>13</v>
@@ -1322,10 +1319,10 @@
     </row>
     <row r="38" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A38" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C38" s="11" t="s">
         <v>13</v>
@@ -1342,10 +1339,10 @@
     </row>
     <row r="39" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A39" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C39" s="11" t="s">
         <v>13</v>
@@ -1362,10 +1359,10 @@
     </row>
     <row r="40" spans="1:6" ht="38.25" customHeight="1" thickBot="1" x14ac:dyDescent="1.1000000000000001">
       <c r="A40" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C40" s="11" t="s">
         <v>13</v>

</xml_diff>